<commit_message>
Perubahan untuk Kaprodi dan update file harus pdf
</commit_message>
<xml_diff>
--- a/template_mahasiswa.xlsx
+++ b/template_mahasiswa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anhar\Documents\Berkas TA Anhar\management_caspstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D108D74-A5D7-43CB-BEB0-A7869A3F16AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1116A13C-91C5-4DD1-ACD7-B0214B365E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -488,7 +488,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>22010100006</v>
+        <v>220101006</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -505,7 +505,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>22010100007</v>
+        <v>220101007</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>22010100008</v>
+        <v>220101008</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
@@ -539,7 +539,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>22010100009</v>
+        <v>220101009</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
@@ -556,7 +556,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
-        <v>22010100010</v>
+        <v>220101010</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
perbaikan pada reset password
</commit_message>
<xml_diff>
--- a/template_mahasiswa.xlsx
+++ b/template_mahasiswa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anhar\Documents\Berkas TA Anhar\management_caspstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1116A13C-91C5-4DD1-ACD7-B0214B365E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{133DDC82-8EAD-4D23-A72C-F329F941D407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>NIM</t>
   </si>
@@ -37,15 +37,9 @@
     <t>📝 Catatan:</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>1. NIM harus unik</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>2. Semua kolom wajib diisi</t>
   </si>
   <si>
@@ -58,12 +52,6 @@
     <t>4. Format: .xlsx atau .xls</t>
   </si>
   <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
     <t>Ahmad Nurul</t>
   </si>
   <si>
@@ -71,12 +59,6 @@
   </si>
   <si>
     <t>Budi Santos</t>
-  </si>
-  <si>
-    <t>Dewi Karo</t>
-  </si>
-  <si>
-    <t>Eko Tio</t>
   </si>
 </sst>
 </file>
@@ -488,27 +470,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>220101006</v>
+        <v>240101999</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="5">
+        <v>2023</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="D2" s="5">
-        <v>2022</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>220101007</v>
+        <v>240101998</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>7</v>
@@ -517,56 +499,39 @@
         <v>2023</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>220101008</v>
+        <v>240101997</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D4" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="5">
-        <v>220101009</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="5">
-        <v>2023</v>
-      </c>
+      <c r="A5" s="5"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="5"/>
       <c r="F5" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="3">
-        <v>220101010</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3">
-        <v>2022</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>